<commit_message>
Regenerate graphs, FINDINGS.xlsx, results.json after adaptive routing update
All outputs refreshed with latest code:
- results.json (includes adaptive τ boundary test data)
- 5 graphs regenerated
- FINDINGS.xlsx 7-sheet workbook regenerated
</commit_message>
<xml_diff>
--- a/FINDINGS.xlsx
+++ b/FINDINGS.xlsx
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>0.484ms</t>
+          <t>0.529ms</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr"/>
@@ -3210,810 +3210,810 @@
     },
     "routing_stats": {
       "overall_accuracy": 0.99875,
-      "avg_time_ms": 0.4843567225032075,
+      "avg_time_ms": 0.5286914124994269,
       "total_samples": 800
     },
     "timing": [
+      0.46790000010332733,
+      0.4603999998380459,
+      0.47309999990829965,
+      0.49190000004273315,
+      0.44809999985773175,
+      0.4515000000537839,
+      0.5487999999331805,
+      0.5460999998376792,
+      0.45660000000680157,
+      0.4546000000118511,
+      0.47459999996135593,
+      0.4441999999471591,
+      0.4449000000477099,
+      0.4458000000795437,
+      0.4804999998668791,
+      0.5851999999322288,
+      0.8035010000639886,
+      0.4765000001043518,
+      0.45560000012301316,
+      0.4621000000497588,
+      0.4651000001558714,
+      0.47730000005685724,
+      0.611899999967136,
+      0.4530999999587948,
+      0.45019999993201054,
+      0.4752999998345331,
+      0.4521000000750064,
+      0.4500000000007276,
+      0.44759999991583754,
+      0.4682000001139386,
+      0.45500000010179065,
+      0.5765999999312044,
+      0.45389999991130026,
+      0.47249999988707714,
+      0.4484999999476713,
+      0.573000000031243,
+      0.6996999998136744,
+      0.6648999999470107,
+      0.8669000001191307,
+      0.7873000001836772,
+      0.520900000083202,
+      0.45760099988001457,
+      0.45119999981579895,
+      0.4738000000088505,
+      0.49130000002151064,
+      0.5593999999291555,
+      0.7368999999926018,
+      0.7130000001325243,
+      0.6547000000409753,
+      0.7528999999522057,
+      0.8617999999387393,
+      0.6757999999535969,
+      0.6834000000708329,
+      0.46590000010837684,
+      0.4526000000169006,
+      0.453599999900689,
+      0.47540000014123507,
+      0.5673999999089574,
+      0.49500000000080036,
+      0.4453999999896041,
+      0.47270000004573376,
+      0.4532000000381231,
+      0.4564000000755186,
+      0.44709999997394334,
+      0.4637000001821434,
+      0.4541999999219115,
+      0.6425009999020403,
+      0.4536000001280627,
+      0.4673000000821048,
+      0.466599999981554,
+      0.44509999997899286,
+      0.4432000000633707,
+      0.44570000000021537,
+      0.48870000000533764,
+      0.8795000001100561,
+      0.7244999999329593,
+      0.47930000005180773,
+      0.44920000004822214,
+      0.4543000000012398,
+      0.45180000006439514,
+      0.4923000001326727,
+      0.6642000000738335,
+      0.4827000000204862,
+      0.6095999999615742,
+      0.4933000000164611,
+      0.48129999981938454,
+      0.48420000007354247,
+      0.5029999999806023,
+      0.5009999999856518,
+      0.6204000001162058,
+      0.4948000000695174,
+      0.527700000020559,
+      0.4844000000048254,
+      0.4849009999361442,
+      0.4954000000907399,
+      0.5074999999123975,
+      0.633900000138965,
+      0.4870000000209984,
+      0.48200000014730904,
+      0.5069999999705033,
+      0.48399999991488585,
+      0.5017999999381573,
+      0.6287999999585736,
+      0.5159000002095127,
+      0.6870999998227489,
+      0.48559999981989677,
+      0.5126000000927888,
+      0.4919999998946878,
+      0.48730000003160967,
+      0.48240000000987493,
+      0.5313999999998487,
+      0.6164999999782594,
+      0.4876000000422209,
+      0.4917000001114502,
+      0.5097999999179592,
+      0.4946999999901891,
+      0.4836999999042746,
+      0.4831999999623804,
+      0.5127000001721171,
+      0.651600999844959,
+      0.5048000000442698,
+      0.48459999993610836,
+      0.5115999999816268,
+      0.48249999986182956,
+      0.48409999999421416,
+      0.4917000001114502,
+      0.5181000001357461,
+      0.6390000000919827,
+      0.48399999991488585,
+      0.5114000000503438,
+      0.5127000001721171,
+      0.48420000007354247,
+      0.4791999999724794,
+      0.6463999998231884,
+      0.5888000000595639,
+      0.48659999993105885,
+      0.4968000000644679,
+      0.5151999998815882,
+      0.48620000006849295,
+      0.506699999959892,
+      0.4823000001579203,
+      0.5105999998704647,
+      0.5827999998473388,
+      0.48500000002604793,
+      0.4813000000467582,
+      0.5112999999710155,
+      0.49040099997910147,
+      0.492600000143284,
+      0.4873999998835643,
+      0.5400000000008731,
+      0.57040000001507,
+      0.47979999999370193,
+      0.4803000001629698,
+      0.5109999999604042,
+      0.4910000000108994,
+      0.48520000018470455,
+      0.48260000016853155,
+      0.5096999998386309,
+      0.5496000001130597,
+      0.48520000018470455,
+      0.4845000000841537,
+      0.5458000000544416,
+      0.48720000017965504,
+      0.702300000057221,
+      0.54679999993823,
+      0.5538999998861982,
+      0.5206999999245454,
+      0.5151999998815882,
+      0.4974000000856904,
+      0.48880000008466595,
+      0.5090999998174084,
+      0.490000000127111,
+      0.4827010000099108,
+      0.5283000000417815,
+      0.50809999993362,
+      0.48079999987749034,
+      0.48139999989871285,
+      0.48919999994723184,
+      0.517100000024584,
+      0.5012999999962631,
+      0.48339999989366333,
+      0.5184000001463573,
+      0.5056999998487299,
+      0.49039999998967687,
+      0.4802000000836415,
+      0.48189999984060705,
+      0.5086999999548425,
+      0.4843000001528708,
+      0.4819000000679807,
+      0.5152999999609165,
+      0.5165000000033615,
+      0.4859000000578817,
+      0.4774999999881402,
+      0.6637999999838939,
+      0.5492999998750747,
+      0.4813000000467582,
+      0.4977999999482563,
+      0.48199999991993536,
+      0.5055999999967753,
+      0.48100000003614696,
+      0.5015000001549197,
+      0.4848999999467196,
+      0.5074000000604428,
+      0.4837999999836029,
+      0.5017999999381573,
+      0.4879000000528322,
+      0.5088999998861254,
+      0.48249999986182956,
+      0.515700000050856,
+      0.49029999991034856,
+      0.5113999998229701,
+      0.48990000004778267,
+      0.5837999999585008,
+      0.48509999987800256,
+      0.5134999998972489,
+      0.48659999993105885,
+      0.48599999990983633,
+      0.4882999999153981,
+      0.5197999998927116,
+      0.5032999999912136,
+      0.5304999999680149,
+      0.5496999999650143,
+      0.4968000000644679,
+      0.4835999998249463,
+      0.7395999998607294,
+      0.5246000000624917,
+      0.48980099995787896,
+      0.5676999999195687,
+      0.4897000001164997,
+      0.5407000001014239,
+      0.49279999984719325,
+      0.4856999998992251,
+      0.4905999999209598,
+      0.5241000001205975,
+      0.48709999987295305,
+      0.5049000001235981,
+      0.4905000000690052,
+      0.5136999998285319,
+      0.4853000000366592,
+      0.4865000000791042,
+      0.5138000001352339,
+      0.5271999998512911,
+      0.48770000012154924,
+      0.5102999998598534,
+      0.4876000000422209,
+      0.5146000000877393,
+      0.5188999998608779,
+      0.49949999993259553,
+      0.48549999996794213,
+      0.5165000000033615,
+      0.513299999965966,
+      0.5406999998740503,
+      0.6343999998534855,
+      0.5499009998857218,
+      0.4893999998785148,
+      0.4922000000533444,
+      0.5163000000720785,
+      0.48830000014277175,
+      0.5023999999593798,
+      0.5188000000089232,
+      0.5122999998548039,
+      0.48509999987800256,
+      0.4827000000204862,
+      0.48289999995176913,
+      0.51989999997204,
+      0.49450000005890615,
+      0.5037999999331078,
+      0.4873999998835643,
+      0.507900000002337,
+      0.5191000000195345,
+      0.492600000143284,
+      0.4905999999209598,
+      0.5144000001564564,
+      0.4883999999947264,
+      0.5034000000705419,
+      0.46739999993405945,
+      0.4747999998926389,
+      0.4532000000381231,
+      0.502899999901274,
+      0.45449999993252277,
+      0.47940000013113604,
+      0.43880099997295474,
+      0.4437999998572195,
+      0.4738000000088505,
+      0.6740999999692576,
+      0.4785999999512569,
+      0.4441999999471591,
+      0.44210000010025396,
+      0.4685999999765045,
+      0.4650999999284977,
+      0.4630999999335472,
+      0.6425999999919441,
+      0.445900000158872,
+      0.6151999998564861,
+      0.449799999842071,
+      0.6619000000682718,
+      0.6729000001541863,
+      0.5315999999311316,
+      0.8442000000741245,
+      0.5148000000190223,
+      0.44470000011642696,
+      0.44520000005832117,
+      0.46009999982743466,
+      0.5165000000033615,
+      0.44819999993706006,
+      0.6275999999161286,
+      0.44980000006944465,
+      0.4681010000240349,
+      0.44709999997394334,
+      0.44100000013713725,
+      0.4418000000896427,
+      0.452199999926961,
+      0.46939999992900994,
+      0.7037999998829036,
+      0.4531000001861685,
+      0.4462999997940642,
+      0.5141999999977998,
+      0.484800000094765,
+      0.44090000005780894,
+      0.5518000000392931,
+      0.48870000000533764,
+      0.5439999999907741,
+      0.44930000012755045,
+      0.48870000000533764,
+      0.5109999999604042,
+      0.5244999999831634,
+      0.5776999998943211,
+      0.44520000005832117,
+      0.49770000009630166,
+      0.5044999998062849,
+      0.48560000004727044,
+      0.44309999998404237,
+      0.46900000006644404,
+      0.44619999994210957,
+      0.4564000000755186,
+      0.4527000000962289,
+      0.4648010001346847,
+      0.5384999999478168,
+      0.4558000000542961,
+      0.49549999994269456,
+      0.480699999798162,
+      0.5803999999898224,
+      0.44129999992037483,
+      0.4449000000477099,
+      0.7005999998455081,
+      0.6115999999565247,
+      0.4794999999830907,
+      0.5667000000357802,
+      0.44670000011137745,
+      0.45030000001133885,
+      0.44150000007903145,
+      0.44879999995828257,
+      0.4682000001139386,
+      0.4897000001164997,
+      0.4484000000957167,
+      0.4432000000633707,
+      0.4655000000184373,
+      0.44959999991078803,
+      0.4744999998820276,
+      0.5148999998709769,
+      0.5955999999969208,
+      0.44449999995777034,
+      0.4578000000492466,
+      0.4520999998476327,
+      0.48000100014178315,
+      0.4822999999305466,
+      0.44040000011591474,
+      0.4698000000189495,
+      0.46219999990171345,
+      0.4773999999088119,
+      0.4993000000013126,
+      0.4453000001376495,
+      0.4453999999896041,
+      0.46629999997094274,
+      0.4397000000153639,
+      0.44150000007903145,
+      0.5449999998745625,
+      0.7055000000946166,
+      0.5077000000710541,
+      0.4415999999309861,
+      0.4507000001012784,
+      0.5436999999801628,
+      0.4392000000734697,
+      0.44720000005327165,
+      0.44200000002092565,
+      0.46419999989666394,
+      0.45019999993201054,
+      0.47530000006190676,
+      0.44299999990471406,
+      0.44000000002597517,
+      0.46960000008766656,
+      0.4519999999956781,
+      0.4894999999578431,
+      0.44150100006845605,
+      0.4999000000225351,
+      0.5013999998482177,
+      0.4437000000052649,
+      0.44150000007903145,
+      0.5129999999553547,
+      0.4930999998578045,
+      0.4519999999956781,
+      0.4467999999633321,
+      1.1202999999113672,
+      0.9729999999308347,
+      1.2927000000217959,
+      0.9390000000166765,
+      0.8173000001079345,
+      0.5767000000105327,
+      0.48360000005231996,
+      0.4500000000007276,
+      0.5155000001195731,
+      0.4437000000052649,
+      0.47459999996135593,
+      0.47679999988758937,
+      0.6344999999328138,
+      0.442901000042184,
+      0.47249999988707714,
+      0.4410999999890919,
+      0.5012999999962631,
+      0.44720000005327165,
+      0.4429000000527594,
+      0.5510999999387423,
+      0.6362999999964813,
+      0.4500000000007276,
+      0.4644999999072752,
+      0.440700000126526,
+      0.4718000000139,
+      0.443300000142699,
+      0.4421999999522086,
+      0.4458999999314983,
+      0.4567999999380845,
+      0.5112000001190609,
+      0.4809999998087733,
+      0.4548000001705077,
+      0.45599999998557905,
+      0.8619000000180677,
+      0.9631000000354106,
+      0.8973999999852822,
+      0.7560000001376466,
+      0.8998000000701722,
+      0.7610010000007605,
+      0.598699999954988,
+      0.5326000000422937,
+      0.45389999991130026,
+      0.4552000000330736,
+      0.4559000001336244,
+      0.4490999999688938,
+      0.4712999998446321,
+      0.4433999999946536,
+      0.4417000000103144,
+      0.445900000158872,
+      0.6224000001111563,
+      0.48310000011042575,
+      0.44439999987844203,
+      0.4725000001144508,
+      0.48040000001492444,
+      0.44520000005832117,
+      0.4831999999623804,
+      0.4449000000477099,
+      0.60910000001968,
+      0.4463000000214379,
+      0.4489000000376109,
+      0.6395999998858315,
+      0.454799999943134,
+      0.4452999999102758,
+      0.4440999998678308,
+      0.4764000000250235,
+      0.5475000000387809,
+      0.4620009999598551,
+      0.4467999999633321,
+      0.47850000009930227,
+      0.45130000012250093,
+      0.448399999868343,
+      0.44819999993706006,
+      0.48670000001038716,
+      0.46789999987595365,
+      0.46169999995981925,
+      0.457399999959307,
+      0.4687000000558328,
+      0.4515000000537839,
+      0.4629000000022643,
+      0.4528999998001382,
+      0.4506000000219501,
+      0.48289999995176913,
+      0.4644999999072752,
+      0.45539999996435654,
+      0.4538000000593456,
+      0.48110000011547527,
+      0.4532000000381231,
+      0.4484999999476713,
+      0.45250000016494596,
+      0.47989999984565657,
+      0.4635999998754414,
+      0.4597999998168234,
+      0.45180000006439514,
+      0.4484000000957167,
+      0.6322000001546257,
+      0.549301000091873,
+      0.4833000000417087,
+      0.46999999995023245,
+      0.463999999965381,
+      0.4521000000750064,
+      0.45240000008561765,
+      0.47459999996135593,
+      0.482200000078592,
+      0.47509999990325014,
+      0.46419999989666394,
+      0.4748999999719672,
+      0.4878999998254585,
+      0.4958000001806795,
+      0.48609999998916464,
+      0.4770999998982006,
+      0.5258999999568914,
+      0.4676999999446707,
+      0.4714000001513341,
+      0.4848999999467196,
+      0.48100000003614696,
+      0.4796999999143736,
+      0.45849999992242374,
+      0.4843000001528708,
+      0.5097000000660046,
+      0.48040000001492444,
+      0.47680000011496304,
+      0.4963000001225737,
+      0.5085000000235596,
+      0.5237010000200826,
+      0.4965999999058113,
+      0.5005999998957122,
+      0.5032000001392589,
+      1.254699999890363,
+      0.4764999998769781,
+      0.4814000001260865,
+      0.5639999999402789,
+      0.4692999998496816,
+      0.49450000005890615,
+      0.5361000000903005,
+      0.4682999999658932,
+      0.4661000000396598,
+      0.4693000000770553,
+      0.497699999868928,
+      0.49290000015389523,
+      0.4698000000189495,
+      0.49860000012813543,
+      0.523399999792673,
+      0.5136999998285319,
+      0.48730000003160967,
+      0.48300000003109744,
+      0.5034999999224965,
+      0.5111999998916872,
+      0.49070000000028813,
+      0.47840000001997396,
+      0.5550999999286432,
+      0.47680100010438764,
+      0.4753999999138614,
+      0.4765000001043518,
+      0.5359000001590175,
+      0.4888999999366206,
+      0.4733000000669563,
+      0.6478000000242901,
+      0.4751000001306238,
+      0.46970000016699487,
+      0.4870000000209984,
+      0.477000000046246,
+      0.517299999955867,
+      0.475600000072518,
+      0.475600000072518,
+      0.5008999999063235,
+      0.5032999999912136,
+      0.4750000000512955,
+      0.4819000000679807,
+      0.4801000000043132,
+      0.5109999999604042,
+      0.5310999999892374,
+      0.48200000014730904,
+      0.5191000000195345,
+      0.504400000181704,
+      0.49300000000584987,
+      0.47109999991334917,
       0.4776000000674685,
-      0.4513000003498746,
-      0.44410000009520445,
-      0.4352999999355234,
-      0.4969000001437962,
-      0.4501000003074296,
-      0.44389999993654783,
-      0.48850000030142837,
-      0.4377000000204134,
-      0.46220000012908713,
-      0.43259999984002206,
-      0.4352999999355234,
-      0.5369000000428059,
-      0.4666999998335086,
-      0.4391000002215151,
-      0.5114999999022984,
-      0.45920000002297456,
+      0.515500999881624,
+      0.474400000030073,
+      0.5138999999871885,
+      0.474400000030073,
+      0.5060000000867149,
+      0.48250000008920324,
+      0.47580000000380096,
+      0.4934999999477441,
+      0.5154999998921994,
+      0.48310000011042575,
+      0.47319999998762796,
+      0.6496000000879576,
+      0.49039999998967687,
+      0.47369999992952216,
+      0.4953000000114116,
+      0.4603999998380459,
+      0.5524000000605156,
+      0.49489999992147204,
+      0.4799999999249849,
+      0.48389999983555754,
+      0.5230999997820618,
+      0.48670000001038716,
+      0.4776000000674685,
+      0.47480000012001256,
+      0.5459999999857246,
+      0.4863999999997759,
+      0.475600000072518,
+      0.5108999998810759,
+      0.4771010001149989,
+      0.47109999991334917,
+      0.47020000010888907,
+      0.4746000001887296,
+      0.5151999998815882,
+      0.47540000014123507,
+      0.47580000000380096,
+      0.4833000000417087,
+      0.5023000001074251,
+      0.4934999999477441,
+      0.4794999999830907,
+      0.47410000001946173,
+      0.5357000000003609,
+      0.4833000000417087,
+      0.6972000001042034,
+      1.4083999999456864,
+      1.3850000000275031,
+      1.2780000001839653,
+      0.9724999999889405,
+      0.8815000001050066,
+      0.8776009999564849,
+      0.7422999999562307,
+      0.5966999999600375,
+      0.5637000001570414,
+      0.7507000000259723,
+      0.6656000000475615,
+      0.5530000000817381,
+      0.7470000000466825,
+      0.7591999999476684,
+      0.7741999997961102,
+      0.4967999998370942,
+      0.6736000000273634,
+      0.7049999999253487,
+      0.9943000000021129,
+      0.5993000002035842,
+      0.559800000019095,
+      0.6290999999691849,
+      0.5877999999484018,
+      0.6034000000454398,
+      0.5609999998341664,
+      0.592099999948914,
+      0.584201000037865,
+      0.5416000001332577,
+      0.5565000001297449,
+      0.5731000001105713,
+      0.6599999999252759,
+      0.5011999999169348,
+      0.5293000001529435,
+      0.5020999999487685,
+      0.7029000000784436,
+      0.5192999999508174,
+      0.5163000000720785,
+      0.6386000000020431,
+      0.518300000067029,
+      0.48310000011042575,
+      0.5131999998866377,
+      0.49390000003768364,
+      0.5103999999391817,
+      0.4822999999305466,
+      0.7624999998370185,
+      0.8675000001403532,
+      0.6467000000611733,
+      0.6300000000010186,
+      0.5780999999842606,
+      0.5450000001019362,
+      0.7039009999516566,
+      0.5525000001398439,
+      0.5595000000084838,
+      0.5252999999356689,
+      0.562400000035268,
+      0.5015999997795006,
+      0.5186000000776403,
+      0.4942000000482949,
+      0.5416999999852123,
+      0.4859000000578817,
+      0.7027999999991152,
+      0.922799999898416,
+      0.8786000000782224,
+      0.5376999999953114,
+      0.611899999967136,
+      0.48659999993105885,
+      0.5126000000927888,
+      0.49810000018624123,
+      0.7861999999931868,
+      0.6700999999793567,
+      1.0647999999946478,
+      0.5266999999093969,
+      1.0131009998985974,
+      0.7193999999799416,
+      0.5117000000609551,
+      0.6731999999374239,
+      0.7851999998820247,
+      0.8789999999407883,
+      0.8391999999730615,
+      0.8803999999145162,
+      0.8940000000166037,
+      0.6130000001576263,
+      0.6769000001440872,
+      0.6464000000505621,
+      0.7984000001215463,
+      0.8478000002014596,
+      0.9179999999560096,
+      0.7794000000558299,
+      0.5066000001079374,
+      0.7120999998733168,
+      0.5295010000736511,
+      0.9024000000863452,
+      0.7327000000714179,
+      0.492600000143284,
+      0.5969000001186942,
+      0.4841999998461688,
+      0.5075999999917258,
+      0.5034000000705419,
+      0.515899999982139,
+      0.505299999986164,
+      0.48289999995176913,
+      0.5155999999715277,
+      0.5163999999240332,
+      0.48250000008920324,
+      0.49909999984265596,
+      0.7093000001532346,
+      0.5372000000534172,
+      0.47889999996186816,
+      0.4959000000326341,
+      0.5581000000347558,
+      0.500099999953818,
+      0.48890000016399426,
+      0.4811999999674299,
+      0.5461000000650529,
+      0.4863999999997759,
+      0.4941009999583912,
+      0.48859999992600933,
+      0.53410000009535,
+      0.4956999998739775,
+      0.4900999999790656,
+      0.8769000000938831,
+      0.49760000001697335,
+      0.4761000000144122,
+      0.4944999998315325,
+      0.4727999998976884,
+      0.4779999999300344,
+      0.46629999997094274,
+      0.4942000000482949,
+      0.5020999999487685,
+      0.4748999999719672,
+      0.4825999999411579,
+      0.5048000000442698,
+      0.4676000000927161,
+      0.469199999997727,
+      0.4650000000765431,
+      0.4655000000184373,
+      0.49119999994218233,
+      0.5113999998229701,
+      0.46789999987595365,
+      0.4630999999335472,
+      0.49130000002151064,
+      0.4676999999446707,
+      0.47369999992952216,
+      0.46020100012356124,
+      0.500099999953818,
+      0.5005999998957122,
+      0.4644999999072752,
+      0.4635999998754414,
+      0.4953000000114116,
+      0.4629000000022643,
+      0.4630000000815926,
+      0.677699999869219,
+      0.5002000000331464,
+      0.48880000008466595,
       0.46999999995023245,
-      0.43679999998857966,
-      0.4370999999991909,
-      1.052099999924394,
-      1.3478000000759494,
-      0.48209999977189,
-      0.5195000003368477,
-      0.447100000201317,
-      0.5150000001776789,
-      0.5377989996304677,
-      0.49510000008012867,
-      0.5035999997744511,
-      0.4831999999623804,
-      0.5154000000402448,
-      0.4612000002452987,
-      0.4926999999952386,
-      0.5017999997107836,
-      0.5801000002065848,
-      0.5240000000412692,
-      0.46419999989666394,
-      0.5781999998362153,
-      0.4639999997380073,
-      0.553300000319723,
-      0.6751999999323743,
-      0.5688999999620137,
-      0.5329000000529049,
-      0.7734999999229331,
-      0.7627999998476298,
-      0.8455000001958979,
-      0.6773000000066531,
-      0.7364999996752886,
-      0.5359000001590175,
-      0.5006000001230859,
-      0.4908999999315711,
-      0.4681999998865649,
-      0.5182999998396554,
-      0.4490000001169392,
-      0.44239999988349155,
-      0.47850000009930227,
-      0.4696999999396212,
-      0.4807990003428131,
-      0.5065000000286091,
-      0.46479999991788645,
-      0.48040000001492444,
-      0.45200000022305176,
-      0.4691999997703533,
-      0.46329999986483017,
-      0.4616000001078646,
-      0.4384999997455452,
-      0.5010999998376064,
-      0.5852000003869762,
-      0.4512000000431726,
-      0.44330000037007267,
-      0.43520000008356874,
-      0.4492999996728031,
-      0.4423000000315369,
-      0.4586999998537067,
-      0.49119999994218233,
-      0.44830000024376204,
-      0.6190000003698515,
-      0.4654999997910636,
-      0.436700000136625,
-      0.445900000158872,
-      0.4567000000861299,
-      0.5112999997436418,
-      0.4517000002124405,
-      0.48599999990983633,
-      0.44350000007398194,
-      0.497699999868928,
-      0.4440999996404571,
-      0.44640000032813987,
-      0.44260000004214817,
-      0.43509999977686675,
-      0.4764000000250235,
-      0.48909999986790353,
-      0.4727999998976884,
-      0.5039000002398097,
-      0.4639989997485827,
-      0.43890000006285845,
-      0.44000000025334884,
-      0.5067000001872657,
-      0.45849999969505006,
-      0.44579999985217,
-      0.46229999998104176,
-      0.44049999996786937,
-      0.4377000000204134,
+      0.47309999990829965,
+      0.4946999999901891,
+      0.46320000001287553,
+      0.46120000001792505,
+      0.4899999998997373,
+      0.49859999990076176,
+      0.47459999996135593,
+      0.4695999998602929,
+      0.4655000000184373,
+      0.4897000001164997,
+      0.462599999991653,
+      0.4650000000765431,
+      0.4637000001821434,
+      0.4911000000902277,
+      0.47819999986131734,
+      0.46689999999216525,
+      0.46650100011902396,
+      0.5541000000448548,
+      0.47270000004573376,
       0.4635999998754414,
-      0.4438000000845932,
-      0.4369999996924889,
-      0.4607999999279855,
-      0.4975000001650187,
-      0.45760000011796365,
-      0.5467000000862754,
-      0.5104000001665554,
-      0.4708999999820662,
-      0.47320000021500164,
-      0.43550000009418,
-      0.4891000003226509,
-      0.4696999999396212,
-      0.48719999995228136,
-      0.45789999967382755,
-      0.44179999986226903,
-      0.47509999967587646,
-      0.444599999809725,
-      0.4337999998824671,
-      0.46750000001338776,
-      0.4442999997991137,
-      0.4612000002452987,
-      0.45279999994818354,
-      0.45760000011796365,
-      0.4543000000012398,
-      0.4700000004049798,
-      0.4741999996440427,
-      0.45589999990625074,
-      0.44559900015883613,
-      0.5423000002338085,
-      0.45200000022305176,
-      0.48659999993105885,
-      0.5175999999664782,
-      0.48850000030142837,
-      0.4444000001058157,
-      0.43779999987236806,
-      0.4414999998516578,
-      0.43759999971371144,
-      0.46229999998104176,
-      0.6438999998863437,
-      0.5063999997219071,
-      0.4368999998405343,
-      0.4774999997607665,
-      0.4410999999890919,
-      0.4334000000199012,
-      0.4358999999567459,
-      0.46579999980167486,
-      0.4920999999740161,
-      0.4423000000315369,
-      0.4377000000204134,
-      0.8149000000230444,
-      0.8364999998775602,
-      0.8833000001686742,
-      0.8290000000670261,
-      0.7906000000730273,
-      0.5658000000039465,
-      0.5160999999134219,
-      0.49560000024939654,
-      0.46960000008766656,
-      0.5004999998163839,
-      0.5610990001514438,
-      0.51050000001851,
-      0.4629999998542189,
-      0.4855999995925231,
-      0.45589999990625074,
-      0.46390000034080003,
-      0.4627999996955623,
-      0.4818999996132334,
-      0.7671999997000967,
-      0.504099999943719,
-      0.4820000003746827,
-      0.4517000002124405,
-      0.47580000000380096,
-      0.44930000012755045,
-      0.44959999968341435,
-      0.4490000001169392,
-      0.46240000028774375,
-      0.48580000020592706,
-      0.4478999999264488,
-      0.44549999984155875,
-      0.44260000004214817,
-      0.47159999985524337,
-      0.4533000001174514,
-      0.4469000000426604,
-      0.444599999809725,
-      0.48540000034336117,
-      0.46440000005532056,
-      0.4919999996673141,
-      0.46619999966424075,
-      0.48659999993105885,
-      0.4490999999688938,
-      0.4428000002008048,
-      0.4467000003387511,
-      0.4656000000977656,
-      0.48160000005736947,
-      0.4469000000426604,
-      0.4428990000633348,
-      0.45649999992747325,
-      0.4654999997910636,
-      0.6203999996614584,
-      0.5247000003691937,
-      0.49479999961477006,
-      0.4564000000755186,
-      0.46280000015030964,
-      0.48969999988912605,
-      0.4571000004034431,
-      0.44930000012755045,
-      0.45959999988554046,
-      0.4695000002357119,
-      0.4506000000219501,
-      0.502899999901274,
-      0.4530999999587948,
-      0.4666999998335086,
-      0.4831999999623804,
-      0.45300000010684016,
-      0.4580999998324842,
-      0.45499999987441697,
-      0.46960000008766656,
-      0.493699999879027,
-      0.44589999970412464,
-      0.4558000000542961,
-      0.47210000002451125,
-      0.44660000003204914,
-      0.4540999998425832,
-      0.48460000016348204,
-      0.5207000003792928,
-      0.45610000006490736,
-      0.46479999991788645,
-      0.44950000028620707,
-      0.45570000020234147,
-      0.4785999999512569,
-      0.4914999999527936,
-      0.4536989999905927,
-      0.6137000000308035,
-      0.47779999977137777,
-      0.5019999998694402,
-      0.5034000000705419,
-      0.45040000031804084,
-      0.47170000016194535,
-      0.44270000034885015,
-      0.46490000022458844,
-      0.44799999977840343,
-      0.46419999989666394,
-      0.46159999965311727,
-      0.4784999996445549,
-      0.47960000028979266,
-      0.45660000023417524,
-      0.4753999996864877,
-      0.4512000000431726,
-      0.4650999999284977,
-      0.44120000029579387,
-      0.4994000000806409,
-      0.4635999998754414,
-      0.4824000002372486,
-      0.44879999995828257,
-      0.47170000016194535,
-      0.4677000001720444,
-      0.44969999999011634,
-      0.46840000004522153,
-      0.44759999991583754,
-      0.47989999984565657,
-      0.4507999997258594,
-      0.4617999998117739,
-      0.47380000023622415,
-      0.4503999998632935,
-      0.46789999987595365,
-      0.4417000000103144,
-      0.44969999999011634,
-      0.8535990000382299,
-      0.46519999978045234,
-      0.45649999992747325,
-      0.47779999977137777,
-      0.4463000000214379,
-      0.4486000002543733,
-      0.44770000022253953,
-      0.47059999997145496,
-      0.5115999997542531,
-      0.46559999964301824,
-      0.4513000003498746,
-      0.4474000002119283,
-      0.4725000003418245,
-      0.44819999993706006,
-      0.44969999999011634,
-      0.44830000024376204,
-      0.46900000006644404,
-      0.4610000000866421,
-      0.4687999999077874,
-      0.45009999985268223,
-      0.4726000001937791,
-      0.4536999999800173,
-      0.4461999997147359,
-      0.4488000004130299,
-      0.44560000014826073,
-      0.48079999987749034,
-      0.4623999998329964,
-      0.44470000011642696,
-      0.47150000000328873,
-      0.4681000000346103,
-      0.4471999995985243,
-      0.4621000002771325,
-      0.45479999971576035,
-      0.6180999998832704,
-      0.4708000001301116,
-      0.452300000233663,
-      0.44919999982084846,
-      0.47479900013058796,
-      0.46939999992900994,
-      0.44410000009520445,
-      0.4455999996935134,
-      0.4444000001058157,
-      0.473000000056345,
-      0.4664000002776447,
-      0.44399999978850246,
-      0.48380000043835025,
-      0.4712999998446321,
-      0.44549999984155875,
-      0.46479999991788645,
-      0.45009999985268223,
-      0.46550000024581095,
-      0.45519999957832624,
-      0.44930000012755045,
-      0.4544999997051491,
-      0.45279999994818354,
-      0.4741000002468354,
-      0.4435999999259366,
-      0.4436999997778912,
-      0.46539999993910897,
-      0.46320000001287553,
-      0.46639999982289737,
-      0.44940000043425243,
-      0.44609999986278126,
-      0.5049999999755528,
-      0.44809999963035807,
-      0.4442999997991137,
-      0.4532000002654968,
-      0.5691999999726249,
-      0.45030000001133885,
-      0.6761999998161627,
-      0.4447999999683816,
-      0.4658000002564222,
-      0.44879999995828257,
-      0.44179999986226903,
-      0.4525989998001023,
-      0.45030000001133885,
-      0.4724000000351225,
-      0.5360000000109721,
-      0.4513999997470819,
-      0.4475000000638829,
-      0.4708999999820662,
-      0.4460000000108266,
-      0.4432999999153253,
-      0.45279999994818354,
-      0.4706999998234096,
-      0.4677000001720444,
-      0.45129999989512726,
-      0.473000000056345,
-      0.4656999999497202,
-      0.4580999998324842,
-      0.4480000002331508,
-      0.4486000002543733,
-      0.4476000003705849,
-      0.47459999996135593,
-      0.462599999991653,
-      0.46419999989666394,
-      0.4484000000957167,
-      0.48659999993105885,
-      0.5581999998867104,
-      0.44879999995828257,
-      0.4465999995773018,
-      0.47409999979208806,
-      0.48659999993105885,
-      0.4515999999057385,
-      0.4451999998309475,
-      0.4436999997778912,
-      0.5043000001023756,
-      0.44570000000021537,
-      0.4883999999947264,
-      0.4446999996616796,
-      0.4650999999284977,
-      0.45969900020281784,
-      0.45240000008561765,
-      0.5004999998163839,
-      0.47309999990829965,
-      0.4473999997571809,
-      0.46010000005480833,
-      0.4546000000118511,
-      0.4785999999512569,
-      0.4959000002600078,
-      0.4512000000431726,
-      0.44579999985217,
-      0.44399999978850246,
-      0.47270000004573376,
-      0.4515999999057385,
-      0.4450000001270382,
-      0.4687000000558328,
-      0.4779999999300344,
-      0.45939999972688383,
-      0.457500000266009,
-      0.6379999999808206,
-      0.5842000000484404,
-      0.4564000000755186,
-      0.46240000028774375,
-      0.46999999995023245,
-      0.4436999997778912,
-      0.4897999997410807,
-      0.4714000001513341,
-      0.4919999996673141,
-      0.47409999979208806,
-      0.4543000000012398,
-      0.4660999998122861,
-      0.46849999989717617,
-      0.4446999996616796,
-      0.4589000000123633,
-      0.46130000009725336,
-      0.48250000008920324,
-      0.4760990000249876,
-      0.46229999998104176,
-      0.4530999999587948,
-      0.45379999983197195,
-      0.48029999970822246,
-      0.47430000040549203,
-      0.47730000005685724,
-      0.47480000012001256,
-      0.48170000036407146,
-      0.4515000000537839,
-      0.47960000028979266,
-      0.45649999992747325,
-      0.4874999999628926,
-      0.4560000002129527,
-      0.4689000002144894,
-      0.5907000004299334,
-      0.46380000003409805,
-      0.4567000000861299,
-      0.462599999991653,
-      0.47900000026857015,
-      0.4517000002124405,
-      0.47110000014072284,
-      0.47170000016194535,
-      0.49770000032367534,
-      0.5036000002291985,
-      0.4604000000654196,
-      0.46229999998104176,
-      0.4799999996976112,
-      0.4641000000447093,
-      0.4469000000426604,
-      0.4629000000022643,
-      0.4997999999432068,
-      0.45129999989512726,
-      0.45490000002246234,
-      0.47110000014072284,
-      0.457500000266009,
-      0.4896000000371714,
-      0.45649899993804866,
-      0.47360000007756753,
-      0.48809999998411513,
-      0.47850000009930227,
-      0.4598999998961517,
-      0.4860000003645837,
-      0.45490000002246234,
-      0.48139999989871285,
-      0.4567999999380845,
-      0.4533000001174514,
-      0.45860000000175205,
-      0.6779000000278756,
-      0.5326999998942483,
-      0.4907999996248691,
-      0.466700000288256,
-      0.49930000022868626,
-      0.4696999999396212,
-      0.46269999984360766,
-      0.49910000007002964,
-      0.4930999998578045,
-      0.45899999986431794,
-      0.45860000000175205,
-      0.4660999998122861,
-      0.4833000002690824,
-      0.4542000001492852,
-      0.4544999997051491,
-      0.4600000002028537,
-      0.4984000001968525,
-      0.4739000000881788,
-      0.4799000003004039,
-      0.4595000000335858,
-      0.477000000046246,
-      0.4611999997905514,
-      0.4650999999284977,
-      0.4608999997799401,
-      0.47389999963343143,
-      0.49029899992092396,
-      0.4714000001513341,
-      0.4650999999284977,
-      0.4733999999189109,
-      0.49179999996340484,
-      0.4616000001078646,
-      0.45610000006490736,
-      0.45649999992747325,
-      1.297300000260293,
-      0.5083000000922766,
-      0.4891000003226509,
-      0.4797000001417473,
-      0.44580000030691735,
-      0.5382999997891602,
-      0.5010999998376064,
-      0.48990000004778267,
-      0.4426999998941028,
-      0.47050000011950033,
-      0.4683999995904742,
-      0.4441999999471591,
-      0.5148999998709769,
-      0.45410000029733055,
-      0.4556999997475941,
-      0.4793000002791814,
-      0.48449999985678005,
-      0.4515000000537839,
-      0.4493999999795051,
-      0.477000000046246,
-      0.46849999989717617,
-      0.44079999997848063,
-      0.4656999999497202,
-      0.4581999996844388,
-      0.48160000005736947,
-      0.45090000003256137,
-      0.4904990000795806,
-      0.4855000001953158,
-      0.4466999998840038,
-      0.47079999967536423,
-      0.45560000035038684,
-      0.5513999999493535,
-      0.5762999999205931,
-      0.47480000012001256,
-      0.4905999999209598,
-      0.4564000000755186,
-      0.47249999988707714,
-      0.45319999981074943,
-      0.4589000000123633,
-      0.45560000035038684,
-      0.5734000001211825,
-      0.45700000009674113,
-      0.44410000009520445,
-      0.4742999999507447,
-      0.4475000000638829,
-      0.4718000000139,
-      0.4417000000103144,
-      0.47249999988707714,
-      0.488499999846681,
-      0.444599999809725,
-      0.4801999998562678,
-      0.475699999697099,
-      0.44350000007398194,
-      0.5234000000200467,
-      0.44100000013713725,
-      0.4629999998542189,
-      0.4708999999820662,
-      0.4484000000957167,
-      0.4704000002675457,
-      0.462700000298355,
-      0.47430000040549203,
-      0.4708000001301116,
-      0.441900000168971,
-      0.4676990001826198,
-      0.44040000011591474,
-      0.6306000000222411,
-      0.5201999997552775,
-      0.44560000014826073,
-      0.4658000002564222,
-      0.4507999997258594,
-      0.4833000002690824,
-      0.47159999985524337,
-      0.44780000007449416,
-      0.4664000002776447,
-      0.4693000000770553,
-      0.43830000004163594,
-      0.44570000000021537,
-      0.4666999998335086,
-      0.467800000023999,
-      0.43500000037965947,
-      0.46769999971729703,
-      0.4349999999249121,
-      0.48299999980372377,
-      0.44060000027457136,
-      0.4646000002139772,
-      0.4382000001896813,
-      0.46900000006644404,
-      0.46459999975922983,
-      0.457399999959307,
-      0.43730000015784753,
-      0.5010000004403992,
-      0.4546000000118511,
-      0.46479999991788645,
-      0.4392000000734697,
-      0.46229999998104176,
-      0.4338999997344217,
-      0.46750000001338776,
-      0.47099999983402085,
-      0.4364999999779684,
-      0.500099999953818,
-      0.6426989998544741,
-      0.48609999976179097,
-      0.46769999971729703,
-      0.43659999982992304,
-      0.4638999998860527,
-      0.43409999989307835,
-      0.46689999999216525,
-      0.4536999999800173,
-      0.43719999985114555,
-      0.4565999997794279,
-      0.43659999982992304,
-      0.4576999999699183,
-      0.49119999994218233,
-      0.4883999999947264,
-      0.43929999992542434,
-      0.4592999998749292,
-      0.4804999998668791,
-      0.4659999999603315,
-      0.4957000001013512,
-      0.5595999996330647,
-      0.4387000003589492,
-      0.4699000000982778,
-      0.4724000000351225,
-      0.44609999986278126,
-      0.5019000000174856,
-      0.44089999983043526,
-      0.4374999998617568,
-      0.49489999992147204,
-      0.4366000002846704,
-      0.5135999999765772,
-      0.5016000000068743,
-      0.43869999990420183,
-      0.49959999978455016,
-      0.46280000015030964,
-      0.7186000002548099,
-      0.46389900035137543,
-      0.4444000001058157,
-      0.4702999999608437,
-      0.4422000001795823,
-      0.43640000012601377,
-      0.4384000003483379,
-      0.5031000000599306,
-      0.4693000000770553,
-      0.4376000001684588,
-      0.4818000002160261,
-      0.440800000433228,
-      0.48470000001543667,
-      0.4722999997284205,
-      0.4393000003801717,
-      0.4963000001225737,
-      0.5019000000174856,
-      0.4401000001053035,
-      0.4446999996616796,
-      0.4386000000522472,
-      0.4662000001189881,
-      0.49699999999575084,
-      0.4496000001381617,
-      0.46369999972739606,
-      0.4934000003231631,
-      0.4685999997491308,
-      0.43779999987236806,
-      0.47779999977137777,
-      0.4358999999567459,
-      0.45920000002297456,
-      0.4488999998102372,
-      0.4963999999745283,
-      0.7275000002664456,
-      0.498899999911373,
-      0.5062999998699524,
-      0.4424999997354462,
-      0.5470000000968867,
-      0.5307000001266715,
-      0.4582990000017162,
-      0.7425999997394683,
-      0.46999999995023245,
-      0.47459999996135593,
-      0.46710000015082187,
-      0.4936000000270724,
-      0.6336999999803083,
-      0.4936000000270724,
-      0.5240999998932239,
-      0.5787999998574378,
-      0.47360000007756753,
-      0.44780000007449416,
-      0.4429000000527594,
-      0.4683000001932669,
-      0.49290000015389523,
-      0.4529999996520928,
-      0.4484999999476713,
-      0.49410000019634026,
-      0.47790000007807976,
-      0.4386000000522472,
-      0.5191999998714891,
-      0.477000000046246,
-      0.4460000000108266,
-      0.4764999998769781,
-      0.43819999973493395,
-      0.4474000002119283,
-      0.6508999999823573,
-      0.5170999997972103,
-      0.4376000001684588,
-      0.43719999985114555,
-      0.4992999997739389,
-      0.44079999997848063,
-      0.4853999998886138,
-      0.4432999999153253,
-      0.5307000001266715,
-      0.4883990000053018,
-      0.43950000008408097,
-      0.4741999996440427,
-      0.4716000003099907,
-      0.4429000000527594,
-      0.49620000027061906,
-      0.4360000002634479,
-      0.4791999999724794,
-      0.48250000008920324,
-      0.4449000002750836,
-      0.44049999996786937,
-      0.4932000001645065,
-      0.7436000000780041,
-      0.6533000000672473,
-      0.5136999998285319,
-      0.7310999999390333,
-      0.6284000000960077,
-      0.5537000001822889,
-      0.4660999998122861,
-      0.44040000011591474,
-      0.4573000001073524,
-      0.6102000002101704,
-      0.6049000003258698,
-      0.4536999999800173,
-      0.5623000001833134,
-      0.5667999998877349,
-      0.546900000244932,
-      0.5727999996452127,
-      0.6420999998226762,
-      0.5500000002029992,
-      0.5348999998204818,
-      0.522499999988213,
-      0.5792990000372811,
-      0.46369999972739606,
-      0.43740000000980217,
-      0.4398000000946922,
-      0.43969999978799024,
-      0.4797000001417473,
-      0.4469000000426604,
-      0.4482000003918074,
-      0.48270000024785986,
-      0.5310000001372828,
-      0.4430000003594614,
-      0.5329999999048596,
-      0.6315000000540749,
-      0.8087999999588646,
-      0.5367999997361039,
-      0.4791999999724794,
-      0.4679999997279083,
-      0.615500000094471,
-      0.5029000003560213,
-      0.4600000002028537,
-      0.5335000000741275,
-      0.4519999997683044,
-      0.44489999982033623,
-      0.4473999997571809,
-      0.46380000003409805,
-      0.44549999984155875,
-      0.4377000000204134,
-      0.441900000168971,
-      0.43719999985114555,
-      0.4895000001852168,
-      0.4831999999623804,
-      0.46729999985473114,
-      0.5390000001170847,
-      0.46619999966424075,
-      0.5223000002843037,
-      0.5432990001281723,
-      0.528900000063004,
-      0.47979999999370193,
-      0.4616000001078646,
-      0.4543000000012398,
-      0.4534999998213607,
-      0.47730000005685724,
-      0.4712999998446321,
-      0.4559000003609981,
-      0.44919999982084846,
-      0.49439999975220417,
-      0.4595000000335858,
-      0.4596999997374951,
-      0.4556999997475941,
-      0.4527000000962289,
-      0.7175000000643195,
-      0.45510000018111896,
-      0.46229999998104176,
-      0.5612999998447776,
-      0.45109999973647064,
-      0.4532000002654968,
-      0.452199999926961,
-      0.47599999970771023,
-      0.46220000012908713,
-      0.4567000000861299,
-      0.4507999997258594,
-      0.48270000024785986
+      0.4672000000027765,
+      0.4841999998461688,
+      0.4963999999745283
     ],
     "global_mse": 0.07361482255381366
   },

</xml_diff>

<commit_message>
Regenerate all outputs after review fixes
</commit_message>
<xml_diff>
--- a/FINDINGS.xlsx
+++ b/FINDINGS.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
     <font>
       <i val="1"/>
@@ -105,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +127,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -677,7 +683,7 @@
           <t>Transformer PPL (overall)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>9.3</t>
         </is>
@@ -694,7 +700,7 @@
           <t>Transformer PPL (code)</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
@@ -711,7 +717,7 @@
           <t>Transformer PPL (math)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>9.6</t>
         </is>
@@ -728,7 +734,7 @@
           <t>Transformer PPL (stories)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>9.9</t>
         </is>
@@ -745,7 +751,7 @@
           <t>Transformer PPL (wiki)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>11.1</t>
         </is>
@@ -779,7 +785,7 @@
           <t>Speed (tok/s)</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>59,492</t>
         </is>
@@ -876,68 +882,78 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Profile-MoE leads on 9 of 12 metrics. Speed + train time are ties.</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>ARCHITECTURAL ADVANTAGES</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>1. SWAPPABLE: Replace any expert → recalibrate profile (seconds) → done. No router retraining.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>2. ZERO learned routing parameters: Router = cos_sim(φ(x), expert_profiles). Pure math.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>3. INTERPRETABLE: Every routing decision is traceable — which expert, why, with what weight.</t>
+          <t>1. SWAPPABLE: Replace any expert → recalibrate profile (seconds) → done. No router retraining.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>4. COLD START: New expert arrives → run on benchmarks → profile ready → joins pool immediately.</t>
+          <t>2. ZERO learned routing parameters: Router = cos_sim(φ(x), expert_profiles). Pure math.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>5. VERSIONED: Profile dimensions are versioned like an API. v1→v2 upgrade = recalibrate all experts.</t>
+          <t>3. INTERPRETABLE: Every routing decision is traceable — which expert, why, with what weight.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>4. COLD START: New expert arrives → run on benchmarks → profile ready → joins pool immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>5. VERSIONED: Profile dimensions are versioned like an API. v1→v2 upgrade = recalibrate all experts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>6. COMPATIBLE: Can adopt DeepSeek innovations (shared experts, fine-grained, bias balancing).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A37:F37"/>
     <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A30:F30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1082,7 +1098,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>0.529ms</t>
+          <t>0.511ms</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr"/>
@@ -1379,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1900,7 +1916,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>After PPL</t>
+          <t>After PPL (profile randomized)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -1937,7 +1953,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>SWAPPED (expected)</t>
+          <t>Profile randomized (not weight swap)</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1970,17 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>~stable</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>~0.5</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>✓ STABLE</t>
+          <t>Weights unchanged</t>
         </is>
       </c>
     </row>
@@ -1981,17 +1997,17 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>~stable</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>~0.6</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>✓ STABLE</t>
+          <t>Weights unchanged</t>
         </is>
       </c>
     </row>
@@ -2008,26 +2024,34 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>~stable</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>~0.6</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>✓ STABLE</t>
+          <t>Weights unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>NOTE: This test randomizes the profile, not the expert weights. A full swap requires replacing FFN weights + recalibrating profile. See mvp.py SwapReport for the complete swap test with weight replacement.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2425,7 +2449,7 @@
       <c r="E25" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Experts continue prediction from hidden state — no context re-reading. This is the architectural win over agentic swarms.</t>
         </is>
@@ -3098,7 +3122,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Full data available in:</t>
         </is>
@@ -3182,7 +3206,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>{
   "evaluation": {
@@ -3210,810 +3234,810 @@
     },
     "routing_stats": {
       "overall_accuracy": 0.99875,
-      "avg_time_ms": 0.5286914124994269,
+      "avg_time_ms": 0.5112844712527931,
       "total_samples": 800
     },
     "timing": [
-      0.46790000010332733,
-      0.4603999998380459,
+      0.4774999997607665,
+      0.6751000000804197,
+      0.4654999997910636,
+      0.5432990001281723,
+      0.5550000000766886,
+      0.48449999985678005,
+      0.5301999999574036,
+      0.5314999998518033,
+      0.5406000000220956,
+      0.5073000002084882,
+      0.5490999997164181,
+      0.5557999998018204,
+      0.5008000002817425,
+      0.5234000000200467,
+      0.4696999999396212,
+      0.46700000029886723,
+      0.832099999570346,
+      0.5522000001292326,
+      0.5188000000089232,
+      0.5298999999467924,
+      0.4951999999320833,
+      0.46109999993859674,
+      0.5510000000867876,
+      0.5153999995854974,
+      0.5264999999781139,
+      0.4646000002139772,
+      0.5399000001489185,
+      0.46999999995023245,
+      0.5564000002777902,
+      0.4548000001705077,
+      0.5134999996698753,
+      0.509299999976065,
+      0.5341999999473046,
+      0.45970000019224244,
+      0.4975000001650187,
+      0.4592999998749292,
+      0.5231000000094355,
+      0.5147990000295977,
+      0.5048000002716435,
+      0.5953999998382642,
+      0.49100000023827306,
+      0.4988000000594184,
+      0.5116000002090004,
+      0.8090000001175213,
+      0.9727999999995518,
+      0.8102000001599663,
+      0.5227999999988242,
+      0.5338999999366933,
+      0.4596000003402878,
+      0.5332000000635162,
+      0.462599999991653,
+      0.49879999960467103,
+      0.6410000000869331,
+      0.4961999998158717,
+      0.5246000000624917,
+      0.4650999999284977,
+      0.5691999999726249,
+      0.48980000019582803,
+      0.582000000122207,
+      0.7200999998531188,
+      0.6647000000157277,
+      0.5086999999548425,
+      0.46169999995981925,
+      0.4809000001841923,
+      0.6868000000395114,
+      0.4602999997587176,
+      0.4984000001968525,
+      0.6494000003840483,
+      0.5221000001256471,
+      0.5080989999441954,
+      0.5095999999866763,
+      1.1304999998174026,
+      0.5737000001317938,
+      0.5852000003869762,
+      0.5188000000089232,
+      0.499000000218075,
+      0.5109000003358233,
+      0.519700000040757,
+      0.4887999998572923,
+      0.47270000004573376,
+      0.46979999979157583,
+      0.5607999996755098,
+      0.4693000000770553,
+      0.5229999997027335,
+      0.49720000015440746,
+      0.5306999996719242,
+      0.4930999998578045,
+      0.4907000002276618,
+      0.5200000000513683,
+      0.5291000002216606,
+      0.5175000001145236,
+      0.46209999982238514,
+      0.49609999996391707,
+      0.5173999998078216,
+      0.5533999997169303,
+      0.4727999998976884,
+      0.5852999997841835,
+      0.48470000001543667,
+      0.4708999999820662,
+      0.5519000001186214,
+      0.656899999739835,
+      0.49040000021705055,
+      0.4837989999941783,
+      0.5980000000818109,
+      0.48339999966628966,
+      0.4582999999911408,
+      0.47829999994064565,
+      0.47360000007756753,
+      0.48079999987749034,
+      0.4602000003615103,
+      0.46090000023468747,
+      0.5270999999993364,
+      0.49859999990076176,
+      0.5015000001549197,
+      0.4589000000123633,
+      0.4830000002584711,
+      0.49370000033377437,
+      0.5458999999063963,
+      0.4582999999911408,
+      0.5577000001721899,
+      0.6382999999914318,
+      0.5516000001080101,
+      0.5250999997770123,
+      0.45610000006490736,
+      0.509400000282767,
+      0.5800000003546302,
+      0.5516999999599648,
+      0.6807999998272862,
+      0.7280999998329207,
+      0.6281000000853965,
+      0.5059000000073866,
+      0.5439000001388195,
+      0.49510000008012867,
+      0.44389999993654783,
+      0.7027000001471606,
+      0.5027000001973647,
+      0.4501990001699596,
+      0.46579999980167486,
+      0.44410000009520445,
+      0.577899999825604,
+      0.44040000011591474,
+      0.5126000000927888,
+      0.5458000000544416,
+      0.5432000002656423,
+      0.44260000004214817,
+      0.47619999986636685,
+      0.4592999998749292,
+      0.5463000002237095,
+      0.4903999997623032,
+      0.541700000212586,
+      0.5227000001468696,
+      0.5315999997037579,
+      0.5817000001115957,
+      0.45799999998052954,
+      0.49250000029132934,
+      0.4764000000250235,
+      0.47940000013113604,
+      0.5291999996188679,
+      0.7061000001158391,
+      0.4961000004186644,
+      0.4505000001699955,
+      0.48230000038529397,
+      0.47079999967536423,
+      0.5258000001049368,
+      0.4585000001497974,
+      0.5317000000104599,
+      0.49370000033377437,
+      0.4633999997167848,
+      0.4543000000012398,
+      0.45550000004368485,
+      0.5191999998714891,
+      0.588299999890296,
+      0.45799899999110494,
+      0.5370999997467152,
+      0.4839999996875122,
+      0.5215999999563792,
+      0.45189999991634977,
+      0.46149999980116263,
+      0.45439999985319446,
+      0.556100000267179,
+      0.45490000002246234,
+      0.4699000000982778,
+      0.4581000002872315,
+      0.48680000008971547,
+      0.493800000185729,
+      0.4629000000022643,
+      0.4644999999072752,
+      0.48100000003614696,
+      0.688099999933911,
+      0.48209999977189,
+      0.46070000007603085,
+      0.4807000000255357,
+      0.4528999998001382,
+      0.475699999697099,
+      0.4604999999173742,
+      0.4849000001740933,
+      0.45479999971576035,
+      0.5227999999988242,
+      0.4619999999704305,
+      0.4772000002049026,
+      0.46750000001338776,
+      0.4536000001280627,
+      0.4564000000755186,
+      0.4751000001306238,
+      0.4538999996839266,
+      0.4523999996308703,
+      0.54679999993823,
+      0.4819000000679807,
+      0.457399999959307,
+      0.4561989999274374,
+      0.45609999961016,
+      0.45399999999062857,
+      0.4819000000679807,
+      0.45379999983197195,
+      0.5734000001211825,
+      0.4567999999380845,
+      0.4791999999724794,
+      0.4652000002351997,
+      0.5280000000311702,
+      1.300800000080926,
+      0.9012000000439002,
+      0.6226999998943938,
+      0.5816999996568484,
+      0.581899999815505,
+      0.628599999799917,
+      0.5836000000272179,
+      0.6803000001127657,
+      0.6509999998343119,
+      0.5368999995880586,
+      0.5243999999038351,
+      0.4855000001953158,
+      0.4936000000270724,
+      0.4718000000139,
+      0.512099999923521,
+      0.6616999999096151,
+      0.5129999999553547,
+      0.47509999967587646,
+      0.47580000000380096,
+      0.4801999998562678,
+      0.5016000000068743,
+      0.4712999998446321,
+      0.6061989997760975,
+      0.4781000002367364,
+      0.5208000002312474,
+      0.5937999999332533,
+      0.9634999996706028,
+      0.5017999997107836,
+      0.4887999998572923,
+      0.6407000000763219,
+      0.4793000002791814,
+      0.47059999997145496,
+      0.4708000001301116,
+      0.4949000003762194,
+      0.4754999999931897,
+      0.4679999997279083,
+      0.49670000043988694,
+      0.5074000000604428,
+      0.4646000002139772,
+      0.46689999999216525,
+      0.4807000000255357,
+      0.4996000002392975,
+      0.46849999989717617,
+      0.4681000000346103,
+      0.46700000029886723,
+      0.5114999999022984,
+      0.47469999981331057,
+      0.46979999979157583,
+      0.46459999975922983,
+      0.4825999999411579,
+      0.4748999999719672,
+      0.48060000017358107,
+      0.46689999999216525,
+      0.47850000009930227,
+      0.574000000142405,
+      0.4658000002564222,
+      0.831199000003835,
+      0.506899999891175,
+      0.4680999995798629,
+      0.46750000001338776,
+      0.47559999984514434,
+      0.5163000000720785,
+      0.48880000031203963,
+      0.4822999999305466,
+      0.4644999999072752,
+      0.4907000002276618,
+      0.5083999999442312,
+      0.4647000000659318,
+      0.46590000010837684,
+      0.5117000000609551,
+      0.4718000000139,
+      0.4679999997279083,
+      0.47440000025744666,
+      0.5372000000534172,
+      0.49319999970975914,
+      0.46840000004522153,
+      0.5031999999118852,
+      0.555999999960477,
+      0.47580000000380096,
+      0.4681000000346103,
+      0.4749999998239218,
+      0.49229999967792537,
+      0.47230000018316787,
+      0.4772999996021099,
+      0.47010000025693444,
+      0.4791000001205248,
+      0.6212000002960849,
+      0.4687999999077874,
+      0.46639999982289737,
+      0.4847999998673913,
+      0.47239999958037515,
+      0.4629000000022643,
+      0.4799000003004039,
+      0.4951989999426587,
+      0.4996999996365048,
+      0.4681000000346103,
+      0.46169999995981925,
+      0.4635999998754414,
+      0.5215999999563792,
+      0.466599999981554,
+      0.4654999997910636,
+      0.46900000006644404,
+      0.505299999986164,
+      0.47480000012001256,
+      0.4752999998345331,
+      0.46619999966424075,
+      0.49239999998462736,
+      0.4696999999396212,
+      0.4666999998335086,
+      0.4953000002387853,
+      0.5121000003782683,
+      0.4693000000770553,
+      0.4652000002351997,
+      0.4635999998754414,
+      0.48680000008971547,
+      0.48299999980372377,
+      0.4647000000659318,
+      0.4674000001614331,
+      0.5375000000640284,
+      0.6640999999945052,
+      0.49919999992198427,
+      0.4702999999608437,
+      0.4623999998329964,
+      0.4604000000654196,
+      0.5016000000068743,
+      0.47869999980321154,
+      0.5294000002322719,
+      0.4735000002256129,
+      0.49560000024939654,
+      0.46619999966424075,
+      0.46239900029831915,
+      0.4619999999704305,
+      0.49489999992147204,
+      0.49279999984719325,
+      0.5240999998932239,
+      0.4652000002351997,
+      0.49770000032367534,
+      0.4718999998658546,
+      0.47249999988707714,
+      0.4636000003301888,
+      0.4901000002064393,
+      0.46769999971729703,
+      0.47929999982443405,
+      0.466700000288256,
+      0.4965000002812303,
+      0.47070000027815695,
+      0.4708999999820662,
+      0.4917000001114502,
+      0.466599999981554,
+      0.4895000001852168,
+      0.7402999999612803,
+      0.5294000002322719,
+      0.5194000000301457,
+      0.4835999998249463,
+      0.47210000002451125,
+      0.5178000001251348,
+      0.5141999999977998,
+      0.4840000001422595,
+      0.5734999999731372,
+      0.49770000032367534,
+      0.47469999981331057,
+      0.47900000026857015,
+      0.4718000000139,
+      0.49970000009125215,
+      0.47829999994064565,
+      0.5194000000301457,
+      0.4902990003756713,
+      0.5074000000604428,
+      0.4794999999830907,
+      0.4733999999189109,
+      0.5203000000619795,
+      1.2713999999505177,
+      1.131600000007893,
+      0.4851000003327499,
+      0.4721999998764659,
+      0.47380000023622415,
+      0.4981999995834485,
+      0.46840000004522153,
+      0.724399999853631,
+      0.6630000002587622,
+      0.47960000028979266,
+      0.5040000000917644,
+      0.47369999992952216,
+      0.5107999995743739,
+      0.46949999978096457,
+      0.4984000001968525,
+      0.5378000000746397,
+      0.47730000005685724,
+      0.4674000001614331,
+      0.5073000002084882,
+      0.4702999999608437,
+      0.5080000000816653,
+      0.47099999983402085,
+      0.492499999836582,
+      0.48219999962384463,
+      0.47139999969658675,
+      0.4700999998021871,
+      0.4948000000695174,
+      0.4905000000690052,
+      0.46649900014017476,
+      0.47360000007756753,
+      0.47989999984565657,
+      0.47989999984565657,
+      0.5384000000958622,
+      0.4677000001720444,
+      0.4698000002463232,
+      0.6121000001257926,
+      1.0098000002471963,
+      0.6683000001430628,
+      0.618199999735225,
+      0.47929999982443405,
+      0.4739000000881788,
+      0.49699999999575084,
+      0.46750000001338776,
+      0.4722999997284205,
+      0.4708000001301116,
+      0.49760000001697335,
+      0.5083999999442312,
+      0.49930000022868626,
+      0.47360000007756753,
+      0.5023999997320061,
+      0.4754999999931897,
+      0.4644999999072752,
+      0.872099999924103,
+      0.5424999999377178,
+      0.4799000003004039,
+      0.4868999999416701,
+      0.5185999998502666,
+      0.4781000002367364,
+      0.4722999997284205,
+      0.4756000002998917,
+      0.5132000001140113,
+      0.5006999999750406,
+      0.4900990002170147,
+      0.47440000025744666,
+      0.4903999997623032,
+      0.46779999956925167,
+      0.6400000002031447,
+      0.500099999953818,
+      0.4915999998047482,
+      0.5286999999043474,
+      0.4714000001513341,
+      0.47059999997145496,
+      0.5012000001443084,
+      0.4718000000139,
+      0.4656000000977656,
+      0.4690999999183987,
+      0.48890000016399426,
+      0.5067000001872657,
+      0.47559999984514434,
+      0.5446999998639512,
+      0.49580000040805317,
+      0.46979999979157583,
+      0.47650000033172546,
+      0.46999999995023245,
+      0.47320000021500164,
+      0.5719999999200809,
+      0.5133999998179206,
+      0.48670000023776083,
+      0.4979000000275846,
+      0.46380000003409805,
+      0.4710000002887682,
+      0.46789999987595365,
+      0.4714000001513341,
+      0.5073000002084882,
+      0.47349999977086554,
+      0.47090000043681357,
+      0.4718999998658546,
+      1.1343989999659243,
+      0.5688999999620137,
+      0.48770000012154924,
+      0.48580000020592706,
+      0.4794999999830907,
+      0.465299999632407,
+      0.500099999953818,
+      0.4720000001725566,
+      0.46590000010837684,
+      0.4679999997279083,
+      0.4997999999432068,
+      0.5289999999149586,
+      0.47099999983402085,
+      0.4721999998764659,
+      0.46789999987595365,
+      0.4914999999527936,
+      0.4770999998982006,
+      0.4801999998562678,
+      0.46710000015082187,
+      0.49699999999575084,
+      0.48890000016399426,
+      0.4994000000806409,
+      0.471900000320602,
+      0.4905000000690052,
+      0.47210000002451125,
+      0.4674000001614331,
+      0.4677000001720444,
+      0.49649999982648296,
+      0.48790000028020586,
+      0.46689999999216525,
+      0.668600000153674,
+      0.5036000002291985,
+      0.5267000001367705,
+      0.47230000018316787,
+      0.4702999999608437,
+      0.49450000005890615,
+      0.5274999998619023,
+      0.4649990000871185,
+      0.47349999977086554,
+      0.5003999999644293,
+      0.4877999999735039,
+      0.46849999989717617,
+      0.5058000001554319,
+      0.488499999846681,
+      0.4812000001948036,
+      0.4778000002261251,
+      0.4670999996960745,
+      0.48349999997299165,
+      0.4708999999820662,
+      0.48940000033326214,
+      0.4749999998239218,
+      0.48699999979362474,
+      0.9310000000368746,
+      0.4687000000558328,
+      0.522399999681511,
+      0.4680999995798629,
+      0.47440000025744666,
+      0.46999999995023245,
+      0.48500000002604793,
+      0.7008000002315384,
+      0.4718000000139,
+      0.651900000320893,
+      0.478099999781989,
+      0.46750000001338776,
+      0.4980999997314939,
+      0.4714000001513341,
+      0.48930000002656016,
+      0.6342000001495762,
+      0.4950999996253813,
+      0.46639999982289737,
+      0.47360000007756753,
+      0.46530000008715433,
+      0.48999900036506006,
+      0.4642999997486186,
+      0.47099999983402085,
+      0.5126999999447435,
+      0.493800000185729,
+      0.47740000036355923,
+      0.4695999996329192,
+      0.49489999992147204,
+      0.4951999999320833,
+      0.4714000001513341,
+      0.46689999999216525,
+      0.5646999998134561,
+      0.4882000002908171,
+      0.48029999970822246,
+      0.46629999997094274,
+      0.5044999998062849,
+      0.46490000022458844,
+      0.4878999998254585,
+      0.46469999961118447,
+      0.5688999999620137,
+      0.7448000001204491,
+      0.505199999679462,
+      0.483299999814335,
+      0.5052000001342094,
+      0.4754999999931897,
+      0.48370000013164827,
+      0.52620000042225,
+      0.5044999998062849,
+      0.4748999999719672,
+      0.5100999997011968,
+      0.5263999996714119,
+      0.5040000000917644,
+      0.4778000002261251,
+      0.4813000000467582,
+      0.48620000006849295,
+      0.5020999997213949,
+      0.5175989999770536,
+      0.4887999998572923,
+      0.5153000001882901,
+      0.5006000001230859,
+      0.48349999997299165,
+      0.5329999999048596,
+      0.5167999997865991,
+      0.5032000003666326,
+      0.5713999998988584,
+      0.47170000016194535,
+      0.4683000001932669,
+      0.4957999999533058,
+      0.4695999996329192,
+      0.4674000001614331,
+      0.5539000003409456,
+      0.7246000000122876,
+      0.47800000038478174,
+      0.47299999960159766,
+      0.46979999979157583,
+      0.4955999997946492,
+      0.4980000003342866,
+      0.6609000001844834,
+      0.5195000003368477,
+      0.47459999996135593,
+      0.4802000003110152,
+      0.4772000002049026,
+      0.49489999992147204,
+      0.4749999998239218,
+      0.4696999999396212,
+      0.5597999997917213,
+      0.6140000000414148,
+      0.5056999998487299,
+      0.47409999979208806,
+      0.5597000003945141,
+      0.49699999999575084,
+      0.4731989997708297,
+      0.4812000001948036,
+      0.5964000001768,
+      0.4973000000063621,
+      0.47580000000380096,
+      0.46920000022510067,
+      0.5162999996173312,
+      0.5080000000816653,
+      0.6074000002627145,
       0.47309999990829965,
-      0.49190000004273315,
-      0.44809999985773175,
-      0.4515000000537839,
-      0.5487999999331805,
-      0.5460999998376792,
-      0.45660000000680157,
-      0.4546000000118511,
-      0.47459999996135593,
-      0.4441999999471591,
-      0.4449000000477099,
-      0.4458000000795437,
-      0.4804999998668791,
-      0.5851999999322288,
-      0.8035010000639886,
-      0.4765000001043518,
-      0.45560000012301316,
-      0.4621000000497588,
-      0.4651000001558714,
-      0.47730000005685724,
-      0.611899999967136,
-      0.4530999999587948,
-      0.45019999993201054,
-      0.4752999998345331,
-      0.4521000000750064,
-      0.4500000000007276,
-      0.44759999991583754,
-      0.4682000001139386,
-      0.45500000010179065,
-      0.5765999999312044,
-      0.45389999991130026,
+      0.5751999997301027,
+      0.661000000036438,
+      0.5292000000736152,
+      0.48040000001492444,
+      0.5387000001064735,
+      0.47210000002451125,
+      0.47199999971780926,
+      0.5853000002389308,
+      0.5145999998603656,
+      0.47480000012001256,
+      0.4722999997284205,
+      0.47230000018316787,
+      0.5007999998269952,
+      0.475699999697099,
+      0.47840000024734763,
+      0.48620000006849295,
+      0.49609999996391707,
+      0.4739999999401334,
+      0.48299999980372377,
+      0.49600000011196244,
+      0.49990000024990877,
+      0.47909999966577743,
+      0.4696999999396212,
+      0.49910000007002964,
+      0.4772000002049026,
+      0.4984990000593825,
+      0.47540000014123507,
+      0.46849999989717617,
+      0.47199999971780926,
+      0.5023000003347988,
+      0.49439999975220417,
+      0.4953000002387853,
+      0.6323999996311613,
+      0.48310000011042575,
+      0.5197999998927116,
+      0.46999999995023245,
+      0.46999999995023245,
+      0.4902000000583939,
       0.47249999988707714,
-      0.4484999999476713,
-      0.573000000031243,
-      0.6996999998136744,
-      0.6648999999470107,
-      0.8669000001191307,
-      0.7873000001836772,
-      0.520900000083202,
-      0.45760099988001457,
-      0.45119999981579895,
-      0.4738000000088505,
-      0.49130000002151064,
-      0.5593999999291555,
-      0.7368999999926018,
-      0.7130000001325243,
-      0.6547000000409753,
-      0.7528999999522057,
-      0.8617999999387393,
-      0.6757999999535969,
-      0.6834000000708329,
-      0.46590000010837684,
-      0.4526000000169006,
-      0.453599999900689,
-      0.47540000014123507,
-      0.5673999999089574,
-      0.49500000000080036,
-      0.4453999999896041,
-      0.47270000004573376,
-      0.4532000000381231,
-      0.4564000000755186,
-      0.44709999997394334,
-      0.4637000001821434,
-      0.4541999999219115,
-      0.6425009999020403,
-      0.4536000001280627,
-      0.4673000000821048,
+      0.4845999997087347,
+      0.47530000028928043,
+      0.5231999998613901,
+      0.46769999971729703,
+      0.47900000026857015,
+      0.47889999996186816,
+      0.5003999999644293,
+      0.46920000022510067,
+      0.4816999999093241,
+      0.47679999988758937,
+      0.5081999997855746,
+      0.4835999998249463,
+      0.47380000023622415,
+      0.49390000003768364,
+      0.4909999997835257,
+      0.46920000022510067,
+      0.48040000001492444,
+      0.5295999999361811,
+      0.4942000000482949,
+      0.46800000018265564,
+      0.4706000004262023,
+      0.47619999986636685,
+      0.4936000000270724,
+      0.5292989999361453,
+      0.6529000002046814,
+      0.8901000001060311,
+      0.4813000000467582,
+      0.4794999999830907,
+      0.5126999999447435,
+      0.5003999999644293,
+      0.4708999999820662,
+      0.4708000001301116,
+      0.5001999998057727,
+      0.5038000003878551,
+      0.46949999978096457,
+      0.46999999995023245,
+      0.5137999996804865,
+      0.5047999998168962,
+      0.4729000002043904,
+      0.4805999997188337,
+      0.48719999995228136,
+      0.4979000000275846,
+      0.4737999997814768,
+      0.5033000002185872,
+      0.47039999981279834,
+      0.5021000001761422,
+      0.4772000002049026,
+      0.471699999707198,
+      0.50020000026052,
+      0.5013999998482177,
+      0.48160000005736947,
+      0.4788000001099135,
+      0.47099999983402085,
+      0.6862999998702435,
+      0.5039000002398097,
+      0.47619999986636685,
+      0.49660000013318495,
+      0.49890000036612037,
+      0.4756989997076744,
+      0.4681999998865649,
+      0.46689999999216525,
+      0.49770000032367534,
+      0.476899999739544,
+      0.46949999978096457,
+      0.5084999997961859,
+      0.4984000001968525,
       0.466599999981554,
-      0.44509999997899286,
-      0.4432000000633707,
-      0.44570000000021537,
-      0.48870000000533764,
-      0.8795000001100561,
-      0.7244999999329593,
-      0.47930000005180773,
-      0.44920000004822214,
-      0.4543000000012398,
-      0.45180000006439514,
-      0.4923000001326727,
-      0.6642000000738335,
-      0.4827000000204862,
-      0.6095999999615742,
-      0.4933000000164611,
-      0.48129999981938454,
-      0.48420000007354247,
-      0.5029999999806023,
-      0.5009999999856518,
-      0.6204000001162058,
-      0.4948000000695174,
-      0.527700000020559,
-      0.4844000000048254,
-      0.4849009999361442,
-      0.4954000000907399,
-      0.5074999999123975,
-      0.633900000138965,
-      0.4870000000209984,
-      0.48200000014730904,
-      0.5069999999705033,
-      0.48399999991488585,
-      0.5017999999381573,
-      0.6287999999585736,
-      0.5159000002095127,
-      0.6870999998227489,
-      0.48559999981989677,
-      0.5126000000927888,
-      0.4919999998946878,
-      0.48730000003160967,
-      0.48240000000987493,
-      0.5313999999998487,
-      0.6164999999782594,
-      0.4876000000422209,
-      0.4917000001114502,
-      0.5097999999179592,
-      0.4946999999901891,
-      0.4836999999042746,
+      0.46249999968495104,
+      0.47130000029937946,
+      0.5041999997956736,
+      0.4650999999284977,
+      0.4644999999072752,
       0.4831999999623804,
-      0.5127000001721171,
-      0.651600999844959,
-      0.5048000000442698,
-      0.48459999993610836,
-      0.5115999999816268,
-      0.48249999986182956,
-      0.48409999999421416,
-      0.4917000001114502,
-      0.5181000001357461,
-      0.6390000000919827,
-      0.48399999991488585,
-      0.5114000000503438,
-      0.5127000001721171,
-      0.48420000007354247,
-      0.4791999999724794,
-      0.6463999998231884,
-      0.5888000000595639,
-      0.48659999993105885,
-      0.4968000000644679,
-      0.5151999998815882,
-      0.48620000006849295,
-      0.506699999959892,
-      0.4823000001579203,
-      0.5105999998704647,
-      0.5827999998473388,
-      0.48500000002604793,
-      0.4813000000467582,
-      0.5112999999710155,
-      0.49040099997910147,
-      0.492600000143284,
-      0.4873999998835643,
-      0.5400000000008731,
-      0.57040000001507,
-      0.47979999999370193,
-      0.4803000001629698,
-      0.5109999999604042,
-      0.4910000000108994,
-      0.48520000018470455,
-      0.48260000016853155,
-      0.5096999998386309,
-      0.5496000001130597,
-      0.48520000018470455,
-      0.4845000000841537,
-      0.5458000000544416,
-      0.48720000017965504,
-      0.702300000057221,
-      0.54679999993823,
-      0.5538999998861982,
-      0.5206999999245454,
-      0.5151999998815882,
-      0.4974000000856904,
-      0.48880000008466595,
-      0.5090999998174084,
-      0.490000000127111,
-      0.4827010000099108,
-      0.5283000000417815,
-      0.50809999993362,
-      0.48079999987749034,
-      0.48139999989871285,
-      0.48919999994723184,
-      0.517100000024584,
-      0.5012999999962631,
-      0.48339999989366333,
-      0.5184000001463573,
-      0.5056999998487299,
-      0.49039999998967687,
-      0.4802000000836415,
-      0.48189999984060705,
-      0.5086999999548425,
-      0.4843000001528708,
-      0.4819000000679807,
-      0.5152999999609165,
-      0.5165000000033615,
-      0.4859000000578817,
-      0.4774999999881402,
-      0.6637999999838939,
-      0.5492999998750747,
-      0.4813000000467582,
-      0.4977999999482563,
-      0.48199999991993536,
-      0.5055999999967753,
-      0.48100000003614696,
-      0.5015000001549197,
-      0.4848999999467196,
-      0.5074000000604428,
-      0.4837999999836029,
-      0.5017999999381573,
-      0.4879000000528322,
-      0.5088999998861254,
-      0.48249999986182956,
-      0.515700000050856,
-      0.49029999991034856,
-      0.5113999998229701,
-      0.48990000004778267,
-      0.5837999999585008,
-      0.48509999987800256,
-      0.5134999998972489,
-      0.48659999993105885,
+      0.5016000000068743,
+      0.46530000008715433,
+      0.45379999983197195,
+      0.5123000000821776,
+      0.4731999997602543,
+      0.4519999997683044,
+      0.4558000000542961,
+      0.5400999998528278,
       0.48599999990983633,
-      0.4882999999153981,
-      0.5197999998927116,
-      0.5032999999912136,
-      0.5304999999680149,
-      0.5496999999650143,
-      0.4968000000644679,
-      0.4835999998249463,
-      0.7395999998607294,
-      0.5246000000624917,
-      0.48980099995787896,
-      0.5676999999195687,
-      0.4897000001164997,
-      0.5407000001014239,
-      0.49279999984719325,
-      0.4856999998992251,
-      0.4905999999209598,
-      0.5241000001205975,
-      0.48709999987295305,
-      0.5049000001235981,
-      0.4905000000690052,
-      0.5136999998285319,
-      0.4853000000366592,
-      0.4865000000791042,
-      0.5138000001352339,
-      0.5271999998512911,
-      0.48770000012154924,
-      0.5102999998598534,
-      0.4876000000422209,
-      0.5146000000877393,
-      0.5188999998608779,
-      0.49949999993259553,
-      0.48549999996794213,
-      0.5165000000033615,
-      0.513299999965966,
-      0.5406999998740503,
-      0.6343999998534855,
-      0.5499009998857218,
-      0.4893999998785148,
-      0.4922000000533444,
-      0.5163000000720785,
-      0.48830000014277175,
-      0.5023999999593798,
-      0.5188000000089232,
-      0.5122999998548039,
-      0.48509999987800256,
-      0.4827000000204862,
-      0.48289999995176913,
-      0.51989999997204,
-      0.49450000005890615,
-      0.5037999999331078,
-      0.4873999998835643,
-      0.507900000002337,
-      0.5191000000195345,
-      0.492600000143284,
-      0.4905999999209598,
-      0.5144000001564564,
+      0.4580999998324842,
+      0.45610000006490736,
+      0.6063000000722241,
+      0.5058000001554319,
+      0.4592999998749292,
+      0.48239999978250125,
+      0.4708999999820662,
+      0.46849999989717617,
+      0.5295000000842265,
+      0.46220000012908713,
+      0.45109999973647064,
+      0.5095999999866763,
+      0.47420000009879004,
+      0.4884989998572564,
+      0.4595000000335858,
+      0.4670999996960745,
+      0.568800000110059,
+      0.483299999814335,
+      0.4490000001169392,
+      0.5135999999765772,
+      0.4745000001094013,
+      0.5254000002423709,
+      0.4524999999375723,
+      0.5487000003085996,
+      0.5206000000725908,
+      0.5407999997260049,
+      0.4963000001225737,
+      0.5845999999110063,
+      0.4698000002463232,
+      0.45899999986431794,
+      0.7457999995494902,
+      0.48110000034284894,
+      0.5903999999645748,
+      0.49770000032367534,
       0.4883999999947264,
-      0.5034000000705419,
-      0.46739999993405945,
-      0.4747999998926389,
-      0.4532000000381231,
-      0.502899999901274,
-      0.45449999993252277,
-      0.47940000013113604,
-      0.43880099997295474,
-      0.4437999998572195,
-      0.4738000000088505,
-      0.6740999999692576,
-      0.4785999999512569,
-      0.4441999999471591,
-      0.44210000010025396,
-      0.4685999999765045,
-      0.4650999999284977,
-      0.4630999999335472,
-      0.6425999999919441,
-      0.445900000158872,
-      0.6151999998564861,
-      0.449799999842071,
-      0.6619000000682718,
-      0.6729000001541863,
-      0.5315999999311316,
-      0.8442000000741245,
-      0.5148000000190223,
-      0.44470000011642696,
-      0.44520000005832117,
-      0.46009999982743466,
-      0.5165000000033615,
-      0.44819999993706006,
-      0.6275999999161286,
-      0.44980000006944465,
-      0.4681010000240349,
-      0.44709999997394334,
-      0.44100000013713725,
-      0.4418000000896427,
-      0.452199999926961,
-      0.46939999992900994,
-      0.7037999998829036,
-      0.4531000001861685,
-      0.4462999997940642,
-      0.5141999999977998,
-      0.484800000094765,
-      0.44090000005780894,
-      0.5518000000392931,
-      0.48870000000533764,
-      0.5439999999907741,
-      0.44930000012755045,
-      0.48870000000533764,
-      0.5109999999604042,
-      0.5244999999831634,
-      0.5776999998943211,
-      0.44520000005832117,
-      0.49770000009630166,
-      0.5044999998062849,
-      0.48560000004727044,
-      0.44309999998404237,
-      0.46900000006644404,
-      0.44619999994210957,
-      0.4564000000755186,
-      0.4527000000962289,
-      0.4648010001346847,
-      0.5384999999478168,
-      0.4558000000542961,
-      0.49549999994269456,
-      0.480699999798162,
-      0.5803999999898224,
-      0.44129999992037483,
-      0.4449000000477099,
-      0.7005999998455081,
-      0.6115999999565247,
-      0.4794999999830907,
-      0.5667000000357802,
-      0.44670000011137745,
-      0.45030000001133885,
-      0.44150000007903145,
-      0.44879999995828257,
-      0.4682000001139386,
-      0.4897000001164997,
-      0.4484000000957167,
-      0.4432000000633707,
-      0.4655000000184373,
-      0.44959999991078803,
-      0.4744999998820276,
-      0.5148999998709769,
-      0.5955999999969208,
-      0.44449999995777034,
-      0.4578000000492466,
-      0.4520999998476327,
-      0.48000100014178315,
-      0.4822999999305466,
-      0.44040000011591474,
-      0.4698000000189495,
-      0.46219999990171345,
-      0.4773999999088119,
-      0.4993000000013126,
-      0.4453000001376495,
-      0.4453999999896041,
-      0.46629999997094274,
-      0.4397000000153639,
-      0.44150000007903145,
-      0.5449999998745625,
-      0.7055000000946166,
-      0.5077000000710541,
-      0.4415999999309861,
-      0.4507000001012784,
-      0.5436999999801628,
-      0.4392000000734697,
-      0.44720000005327165,
-      0.44200000002092565,
-      0.46419999989666394,
-      0.45019999993201054,
-      0.47530000006190676,
-      0.44299999990471406,
-      0.44000000002597517,
-      0.46960000008766656,
-      0.4519999999956781,
-      0.4894999999578431,
-      0.44150100006845605,
-      0.4999000000225351,
-      0.5013999998482177,
-      0.4437000000052649,
-      0.44150000007903145,
-      0.5129999999553547,
-      0.4930999998578045,
-      0.4519999999956781,
-      0.4467999999633321,
-      1.1202999999113672,
-      0.9729999999308347,
-      1.2927000000217959,
-      0.9390000000166765,
-      0.8173000001079345,
-      0.5767000000105327,
-      0.48360000005231996,
-      0.4500000000007276,
-      0.5155000001195731,
-      0.4437000000052649,
-      0.47459999996135593,
-      0.47679999988758937,
-      0.6344999999328138,
-      0.442901000042184,
-      0.47249999988707714,
-      0.4410999999890919,
-      0.5012999999962631,
-      0.44720000005327165,
-      0.4429000000527594,
-      0.5510999999387423,
-      0.6362999999964813,
-      0.4500000000007276,
-      0.4644999999072752,
-      0.440700000126526,
-      0.4718000000139,
-      0.443300000142699,
-      0.4421999999522086,
-      0.4458999999314983,
-      0.4567999999380845,
-      0.5112000001190609,
-      0.4809999998087733,
-      0.4548000001705077,
-      0.45599999998557905,
-      0.8619000000180677,
-      0.9631000000354106,
-      0.8973999999852822,
-      0.7560000001376466,
-      0.8998000000701722,
-      0.7610010000007605,
-      0.598699999954988,
-      0.5326000000422937,
-      0.45389999991130026,
-      0.4552000000330736,
-      0.4559000001336244,
-      0.4490999999688938,
-      0.4712999998446321,
-      0.4433999999946536,
-      0.4417000000103144,
-      0.445900000158872,
-      0.6224000001111563,
-      0.48310000011042575,
-      0.44439999987844203,
-      0.4725000001144508,
-      0.48040000001492444,
-      0.44520000005832117,
-      0.4831999999623804,
-      0.4449000000477099,
-      0.60910000001968,
-      0.4463000000214379,
-      0.4489000000376109,
-      0.6395999998858315,
-      0.454799999943134,
-      0.4452999999102758,
-      0.4440999998678308,
-      0.4764000000250235,
-      0.5475000000387809,
-      0.4620009999598551,
-      0.4467999999633321,
-      0.47850000009930227,
-      0.45130000012250093,
-      0.448399999868343,
-      0.44819999993706006,
-      0.48670000001038716,
-      0.46789999987595365,
-      0.46169999995981925,
-      0.457399999959307,
-      0.4687000000558328,
-      0.4515000000537839,
-      0.4629000000022643,
-      0.4528999998001382,
-      0.4506000000219501,
-      0.48289999995176913,
-      0.4644999999072752,
-      0.45539999996435654,
-      0.4538000000593456,
-      0.48110000011547527,
-      0.4532000000381231,
-      0.4484999999476713,
-      0.45250000016494596,
-      0.47989999984565657,
-      0.4635999998754414,
-      0.4597999998168234,
-      0.45180000006439514,
-      0.4484000000957167,
-      0.6322000001546257,
-      0.549301000091873,
-      0.4833000000417087,
-      0.46999999995023245,
-      0.463999999965381,
-      0.4521000000750064,
-      0.45240000008561765,
-      0.47459999996135593,
-      0.482200000078592,
-      0.47509999990325014,
-      0.46419999989666394,
-      0.4748999999719672,
-      0.4878999998254585,
-      0.4958000001806795,
-      0.48609999998916464,
-      0.4770999998982006,
-      0.5258999999568914,
-      0.4676999999446707,
-      0.4714000001513341,
-      0.4848999999467196,
-      0.48100000003614696,
-      0.4796999999143736,
-      0.45849999992242374,
-      0.4843000001528708,
-      0.5097000000660046,
-      0.48040000001492444,
-      0.47680000011496304,
-      0.4963000001225737,
-      0.5085000000235596,
-      0.5237010000200826,
-      0.4965999999058113,
-      0.5005999998957122,
-      0.5032000001392589,
-      1.254699999890363,
-      0.4764999998769781,
-      0.4814000001260865,
-      0.5639999999402789,
-      0.4692999998496816,
-      0.49450000005890615,
-      0.5361000000903005,
-      0.4682999999658932,
-      0.4661000000396598,
-      0.4693000000770553,
-      0.497699999868928,
-      0.49290000015389523,
-      0.4698000000189495,
-      0.49860000012813543,
-      0.523399999792673,
-      0.5136999998285319,
-      0.48730000003160967,
-      0.48300000003109744,
-      0.5034999999224965,
-      0.5111999998916872,
-      0.49070000000028813,
-      0.47840000001997396,
-      0.5550999999286432,
-      0.47680100010438764,
-      0.4753999999138614,
-      0.4765000001043518,
-      0.5359000001590175,
-      0.4888999999366206,
-      0.4733000000669563,
-      0.6478000000242901,
-      0.4751000001306238,
-      0.46970000016699487,
-      0.4870000000209984,
-      0.477000000046246,
-      0.517299999955867,
-      0.475600000072518,
-      0.475600000072518,
-      0.5008999999063235,
-      0.5032999999912136,
-      0.4750000000512955,
-      0.4819000000679807,
-      0.4801000000043132,
-      0.5109999999604042,
-      0.5310999999892374,
-      0.48200000014730904,
-      0.5191000000195345,
-      0.504400000181704,
-      0.49300000000584987,
-      0.47109999991334917,
-      0.4776000000674685,
-      0.515500999881624,
-      0.474400000030073,
-      0.5138999999871885,
-      0.474400000030073,
-      0.5060000000867149,
-      0.48250000008920324,
-      0.47580000000380096,
-      0.4934999999477441,
-      0.5154999998921994,
-      0.48310000011042575,
-      0.47319999998762796,
-      0.6496000000879576,
-      0.49039999998967687,
-      0.47369999992952216,
-      0.4953000000114116,
-      0.4603999998380459,
-      0.5524000000605156,
-      0.49489999992147204,
-      0.4799999999249849,
-      0.48389999983555754,
-      0.5230999997820618,
-      0.48670000001038716,
-      0.4776000000674685,
-      0.47480000012001256,
-      0.5459999999857246,
-      0.4863999999997759,
-      0.475600000072518,
-      0.5108999998810759,
-      0.4771010001149989,
-      0.47109999991334917,
-      0.47020000010888907,
-      0.4746000001887296,
-      0.5151999998815882,
-      0.47540000014123507,
-      0.47580000000380096,
-      0.4833000000417087,
-      0.5023000001074251,
-      0.4934999999477441,
-      0.4794999999830907,
-      0.47410000001946173,
-      0.5357000000003609,
-      0.4833000000417087,
-      0.6972000001042034,
-      1.4083999999456864,
-      1.3850000000275031,
-      1.2780000001839653,
-      0.9724999999889405,
-      0.8815000001050066,
-      0.8776009999564849,
-      0.7422999999562307,
-      0.5966999999600375,
-      0.5637000001570414,
-      0.7507000000259723,
-      0.6656000000475615,
-      0.5530000000817381,
-      0.7470000000466825,
-      0.7591999999476684,
-      0.7741999997961102,
-      0.4967999998370942,
-      0.6736000000273634,
-      0.7049999999253487,
-      0.9943000000021129,
-      0.5993000002035842,
-      0.559800000019095,
-      0.6290999999691849,
-      0.5877999999484018,
-      0.6034000000454398,
-      0.5609999998341664,
-      0.592099999948914,
-      0.584201000037865,
-      0.5416000001332577,
-      0.5565000001297449,
-      0.5731000001105713,
-      0.6599999999252759,
-      0.5011999999169348,
-      0.5293000001529435,
-      0.5020999999487685,
-      0.7029000000784436,
-      0.5192999999508174,
-      0.5163000000720785,
-      0.6386000000020431,
-      0.518300000067029,
-      0.48310000011042575,
-      0.5131999998866377,
-      0.49390000003768364,
-      0.5103999999391817,
-      0.4822999999305466,
-      0.7624999998370185,
-      0.8675000001403532,
-      0.6467000000611733,
-      0.6300000000010186,
-      0.5780999999842606,
-      0.5450000001019362,
-      0.7039009999516566,
-      0.5525000001398439,
-      0.5595000000084838,
-      0.5252999999356689,
-      0.562400000035268,
-      0.5015999997795006,
-      0.5186000000776403,
-      0.4942000000482949,
-      0.5416999999852123,
-      0.4859000000578817,
-      0.7027999999991152,
-      0.922799999898416,
-      0.8786000000782224,
-      0.5376999999953114,
-      0.611899999967136,
-      0.48659999993105885,
-      0.5126000000927888,
-      0.49810000018624123,
-      0.7861999999931868,
-      0.6700999999793567,
-      1.0647999999946478,
-      0.5266999999093969,
-      1.0131009998985974,
-      0.7193999999799416,
-      0.5117000000609551,
-      0.6731999999374239,
-      0.7851999998820247,
-      0.8789999999407883,
-      0.8391999999730615,
-      0.8803999999145162,
-      0.8940000000166037,
-      0.6130000001576263,
-      0.6769000001440872,
-      0.6464000000505621,
-      0.7984000001215463,
-      0.8478000002014596,
-      0.9179999999560096,
-      0.7794000000558299,
-      0.5066000001079374,
-      0.7120999998733168,
-      0.5295010000736511,
-      0.9024000000863452,
-      0.7327000000714179,
-      0.492600000143284,
-      0.5969000001186942,
-      0.4841999998461688,
-      0.5075999999917258,
-      0.5034000000705419,
-      0.515899999982139,
-      0.505299999986164,
-      0.48289999995176913,
-      0.5155999999715277,
-      0.5163999999240332,
-      0.48250000008920324,
-      0.49909999984265596,
-      0.7093000001532346,
-      0.5372000000534172,
-      0.47889999996186816,
-      0.4959000000326341,
-      0.5581000000347558,
-      0.500099999953818,
-      0.48890000016399426,
-      0.4811999999674299,
-      0.5461000000650529,
-      0.4863999999997759,
-      0.4941009999583912,
-      0.48859999992600933,
-      0.53410000009535,
-      0.4956999998739775,
-      0.4900999999790656,
-      0.8769000000938831,
-      0.49760000001697335,
-      0.4761000000144122,
-      0.4944999998315325,
-      0.4727999998976884,
-      0.4779999999300344,
-      0.46629999997094274,
-      0.4942000000482949,
-      0.5020999999487685,
-      0.4748999999719672,
-      0.4825999999411579,
-      0.5048000000442698,
-      0.4676000000927161,
-      0.469199999997727,
-      0.4650000000765431,
-      0.4655000000184373,
-      0.49119999994218233,
-      0.5113999998229701,
-      0.46789999987595365,
-      0.4630999999335472,
-      0.49130000002151064,
-      0.4676999999446707,
-      0.47369999992952216,
-      0.46020100012356124,
-      0.500099999953818,
-      0.5005999998957122,
-      0.4644999999072752,
-      0.4635999998754414,
-      0.4953000000114116,
-      0.4629000000022643,
-      0.4630000000815926,
-      0.677699999869219,
-      0.5002000000331464,
-      0.48880000008466595,
-      0.46999999995023245,
-      0.47309999990829965,
-      0.4946999999901891,
-      0.46320000001287553,
-      0.46120000001792505,
-      0.4899999998997373,
-      0.49859999990076176,
-      0.47459999996135593,
-      0.4695999998602929,
-      0.4655000000184373,
-      0.4897000001164997,
-      0.462599999991653,
-      0.4650000000765431,
-      0.4637000001821434,
-      0.4911000000902277,
-      0.47819999986131734,
-      0.46689999999216525,
-      0.46650100011902396,
-      0.5541000000448548,
-      0.47270000004573376,
-      0.4635999998754414,
-      0.4672000000027765,
-      0.4841999998461688,
-      0.4963999999745283
+      0.4742999999507447,
+      0.5464000000756641,
+      0.4947000002175628,
+      0.5179999998290441
     ],
     "global_mse": 0.07361482255381366
   },
@@ -4157,7 +4181,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>{
   "learned_router": {

</xml_diff>